<commit_message>
feat: add mobile name nomination requests
</commit_message>
<xml_diff>
--- a/outputs/019ff074-0242-7193-82b3-fe7027689c8c/صلاحيات_النظام.xlsx
+++ b/outputs/019ff074-0242-7193-82b3-fe7027689c8c/صلاحيات_النظام.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كل الصلاحيات" sheetId="1" r:id="R58c2c6e7fec44a48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص حسب الوحدة" sheetId="2" r:id="R64e260c2b07147c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اختبار الأدوار" sheetId="3" r:id="Rcfceb62f647a4ee8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اعتماد الزبائن" sheetId="4" r:id="Raf33c7d455234ef8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="كل الصلاحيات" sheetId="1" r:id="R9159ecccbcf74a31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملخص حسب الوحدة" sheetId="2" r:id="R3b22dcdfb16a43e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اختبار الأدوار" sheetId="3" r:id="R2a6b69d48d284179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اعتماد الزبائن" sheetId="4" r:id="Rec2433b277834833"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -117,7 +117,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="40">
+  <x:fills count="41">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -314,6 +314,11 @@
         <x:fgColor rgb="FFC6EFCE"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6EFCE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -349,7 +354,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="121">
+  <x:cellXfs count="124">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -639,6 +644,11 @@
     <x:xf numFmtId="0" fontId="14" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="18" fillId="39" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="10" fillId="39" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -10447,6 +10457,206 @@
         <x:v>بوابة الهاتف تتطلب telemarketing.calls.create وتتحقق من فرع المستفيد والجهاز.</x:v>
       </x:c>
     </x:row>
+    <x:row r="164">
+      <x:c r="A164" s="123" t="n">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="B164" s="123"/>
+      <x:c r="C164" s="123" t="str">
+        <x:v>طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="D164" s="123" t="str">
+        <x:v>name_nomination</x:v>
+      </x:c>
+      <x:c r="E164" s="123" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F164" s="123" t="str">
+        <x:v>view</x:v>
+      </x:c>
+      <x:c r="G164" s="123" t="str">
+        <x:v>عرض طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="H164" s="123" t="str">
+        <x:v>name_nomination.view</x:v>
+      </x:c>
+      <x:c r="I164" s="123" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J164" s="123" t="n">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="K164" s="123" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L164" s="123"/>
+      <x:c r="M164" s="123" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="N164" s="123" t="str">
+        <x:v>صلاحية مركزية بنطاق GLOBAL فقط؛ لا يعتمد القرار على فرع الطلب.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" s="123" t="n">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="B165" s="123"/>
+      <x:c r="C165" s="123" t="str">
+        <x:v>طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="D165" s="123" t="str">
+        <x:v>name_nomination</x:v>
+      </x:c>
+      <x:c r="E165" s="123" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F165" s="123" t="str">
+        <x:v>review</x:v>
+      </x:c>
+      <x:c r="G165" s="123" t="str">
+        <x:v>مراجعة طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="H165" s="123" t="str">
+        <x:v>name_nomination.review</x:v>
+      </x:c>
+      <x:c r="I165" s="123" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J165" s="123" t="n">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="K165" s="123" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L165" s="123"/>
+      <x:c r="M165" s="123" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="N165" s="123" t="str">
+        <x:v>صلاحية مركزية بنطاق GLOBAL فقط؛ لا يعتمد القرار على فرع الطلب.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" s="123" t="n">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="B166" s="123"/>
+      <x:c r="C166" s="123" t="str">
+        <x:v>طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="D166" s="123" t="str">
+        <x:v>name_nomination</x:v>
+      </x:c>
+      <x:c r="E166" s="123" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F166" s="123" t="str">
+        <x:v>decide</x:v>
+      </x:c>
+      <x:c r="G166" s="123" t="str">
+        <x:v>حسم طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="H166" s="123" t="str">
+        <x:v>name_nomination.decide</x:v>
+      </x:c>
+      <x:c r="I166" s="123" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J166" s="123" t="n">
+        <x:v>294</x:v>
+      </x:c>
+      <x:c r="K166" s="123" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L166" s="123"/>
+      <x:c r="M166" s="123" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="N166" s="123" t="str">
+        <x:v>صلاحية مركزية بنطاق GLOBAL فقط؛ لا يعتمد القرار على فرع الطلب.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" s="123" t="n">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="B167" s="123"/>
+      <x:c r="C167" s="123" t="str">
+        <x:v>طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="D167" s="123" t="str">
+        <x:v>name_nomination</x:v>
+      </x:c>
+      <x:c r="E167" s="123" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F167" s="123" t="str">
+        <x:v>resolve_escalation</x:v>
+      </x:c>
+      <x:c r="G167" s="123" t="str">
+        <x:v>فك تصعيد طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="H167" s="123" t="str">
+        <x:v>name_nomination.resolve_escalation</x:v>
+      </x:c>
+      <x:c r="I167" s="123" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J167" s="123" t="n">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="K167" s="123" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L167" s="123"/>
+      <x:c r="M167" s="123" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="N167" s="123" t="str">
+        <x:v>صلاحية مركزية بنطاق GLOBAL فقط؛ لا يعتمد القرار على فرع الطلب.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" s="123" t="n">
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="B168" s="123"/>
+      <x:c r="C168" s="123" t="str">
+        <x:v>طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="D168" s="123" t="str">
+        <x:v>name_nomination</x:v>
+      </x:c>
+      <x:c r="E168" s="123" t="str">
+        <x:v>service_requests</x:v>
+      </x:c>
+      <x:c r="F168" s="123" t="str">
+        <x:v>archive</x:v>
+      </x:c>
+      <x:c r="G168" s="123" t="str">
+        <x:v>أرشفة طلبات ترشيح الأسماء</x:v>
+      </x:c>
+      <x:c r="H168" s="123" t="str">
+        <x:v>name_nomination.archive</x:v>
+      </x:c>
+      <x:c r="I168" s="123" t="str">
+        <x:v>عام (كل الفروع)</x:v>
+      </x:c>
+      <x:c r="J168" s="123" t="n">
+        <x:v>296</x:v>
+      </x:c>
+      <x:c r="K168" s="123" t="str">
+        <x:v>❌</x:v>
+      </x:c>
+      <x:c r="L168" s="123"/>
+      <x:c r="M168" s="123" t="str">
+        <x:v>مضاف</x:v>
+      </x:c>
+      <x:c r="N168" s="123" t="str">
+        <x:v>صلاحية مركزية بنطاق GLOBAL فقط؛ لا يعتمد القرار على فرع الطلب.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>